<commit_message>
fix PX3155 MedPhys availability error
</commit_message>
<xml_diff>
--- a/AssessmentSchedule_2627.xlsx
+++ b/AssessmentSchedule_2627.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cf-my.sharepoint.com/personal/northce_cardiff_ac_uk/Documents/Documents/Cardiff/DUGS/Assessments/Schedule Modelling/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1968" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0B50F5B-5B0D-4468-862C-2FC2AB068C54}"/>
+  <xr:revisionPtr revIDLastSave="1969" documentId="8_{F30C7968-F540-46E6-A81C-665FBDA0D3DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82417EF7-A2EA-4B8F-8F87-9925D190BB89}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" activeTab="2" xr2:uid="{A20BCC1C-F123-4C76-9181-B345A7D760BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessments" sheetId="1" r:id="rId1"/>
@@ -1627,29 +1627,86 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="0" tint="-0.249977111117893"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1667,13 +1724,8 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1691,10 +1743,11 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1715,6 +1768,32 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -1739,30 +1818,7 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
@@ -1787,14 +1843,8 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1812,14 +1862,14 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
+          <bgColor indexed="65"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
       <font>
@@ -1837,14 +1887,14 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="164" formatCode="0.000"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
       <font>
@@ -1862,136 +1912,48 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -2042,132 +2004,6 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="1" formatCode="0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -2720,6 +2556,178 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color auto="1"/>
@@ -2807,6 +2815,81 @@
         <top/>
         <bottom/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
       <font>
@@ -3424,6 +3507,61 @@
         <name val="Calibri (Body)"/>
         <scheme val="none"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
@@ -3443,6 +3581,171 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="1" formatCode="0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri (Body)"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -3533,309 +3836,6 @@
         <bottom/>
       </border>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Calibri (Body)"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3850,56 +3850,56 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FA69A777-C149-48BD-B248-35F32F0AC920}" name="Table1" displayName="Table1" ref="A1:AL184" totalsRowShown="0" headerRowDxfId="94" dataDxfId="92" headerRowBorderDxfId="93" tableBorderDxfId="91" totalsRowBorderDxfId="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FA69A777-C149-48BD-B248-35F32F0AC920}" name="Table1" displayName="Table1" ref="A1:AL184" totalsRowShown="0" headerRowDxfId="113" dataDxfId="111" headerRowBorderDxfId="112" tableBorderDxfId="110" totalsRowBorderDxfId="109">
   <autoFilter ref="A1:AL184" xr:uid="{FA69A777-C149-48BD-B248-35F32F0AC920}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AI155">
     <sortCondition ref="A1:A155"/>
   </sortState>
   <tableColumns count="38">
-    <tableColumn id="1" xr3:uid="{7078548A-F011-4851-AB36-1F04238FA2FE}" name="Module Code" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{D2290F36-B8B3-427A-AEFE-45FD22901411}" name="Module Title" dataDxfId="17">
+    <tableColumn id="1" xr3:uid="{7078548A-F011-4851-AB36-1F04238FA2FE}" name="Module Code" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{D2290F36-B8B3-427A-AEFE-45FD22901411}" name="Module Title" dataDxfId="107">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Table1[[#This Row],[Module Code]],Table2[Module Code],Table2[Module Title])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="33" xr3:uid="{B83E0E3E-2B28-42F1-BC64-5D7177EC4229}" name="CA Weight" dataDxfId="27"/>
-    <tableColumn id="34" xr3:uid="{AEA2048C-138D-450A-BE52-3FCBDE03C67D}" name="Credits" dataDxfId="25"/>
-    <tableColumn id="3" xr3:uid="{31165455-2AA3-4532-A0A0-C942837C0F79}" name="CA type" dataDxfId="13"/>
-    <tableColumn id="30" xr3:uid="{82DD5B5B-C808-4E6E-849C-7A03DC6D0B69}" name="Description" dataDxfId="26"/>
-    <tableColumn id="36" xr3:uid="{A7BF30F6-C808-4B8F-B3FF-9FAF20E2145A}" name="Summative" dataDxfId="89"/>
-    <tableColumn id="37" xr3:uid="{68E504F9-116C-43AB-BCC6-3BB48B0860D2}" name="Day of Week" dataDxfId="88"/>
-    <tableColumn id="16" xr3:uid="{E6637FEB-7F23-45F0-99D2-96D20DD2DAEF}" name="Duration" dataDxfId="24"/>
-    <tableColumn id="31" xr3:uid="{FD1E9614-3960-4F72-BD42-711A4CC7BBA0}" name="Nominal Hours" dataDxfId="22">
+    <tableColumn id="33" xr3:uid="{B83E0E3E-2B28-42F1-BC64-5D7177EC4229}" name="CA Weight" dataDxfId="106"/>
+    <tableColumn id="34" xr3:uid="{AEA2048C-138D-450A-BE52-3FCBDE03C67D}" name="Credits" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{31165455-2AA3-4532-A0A0-C942837C0F79}" name="CA type" dataDxfId="104"/>
+    <tableColumn id="30" xr3:uid="{82DD5B5B-C808-4E6E-849C-7A03DC6D0B69}" name="Description" dataDxfId="103"/>
+    <tableColumn id="36" xr3:uid="{A7BF30F6-C808-4B8F-B3FF-9FAF20E2145A}" name="Summative" dataDxfId="102"/>
+    <tableColumn id="37" xr3:uid="{68E504F9-116C-43AB-BCC6-3BB48B0860D2}" name="Day of Week" dataDxfId="101"/>
+    <tableColumn id="16" xr3:uid="{E6637FEB-7F23-45F0-99D2-96D20DD2DAEF}" name="Duration" dataDxfId="100"/>
+    <tableColumn id="31" xr3:uid="{FD1E9614-3960-4F72-BD42-711A4CC7BBA0}" name="Nominal Hours" dataDxfId="99">
       <calculatedColumnFormula>IFERROR(AVERAGEIF(Table1[[#This Row],[Autumn Week 1]:[Spring Exams]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Exams]])*4*Table1[[#This Row],[Credits]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="32" xr3:uid="{E11C773A-511F-4D25-8636-C56C5B61ED90}" name="Hours" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{04E38F13-8347-412C-866C-6EFE6796253C}" name="Autumn Week 1" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{254D6A24-FC1B-44C7-A3DF-52DA2A250D31}" name="Autumn Week 2" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{9EB326C3-772E-4E56-89FB-BA3A00291293}" name="Autumn Week 3" dataDxfId="85"/>
-    <tableColumn id="7" xr3:uid="{94BC6C78-5A89-4267-B1C1-BFA70E5A9F34}" name="Autumn Week 4" dataDxfId="84"/>
-    <tableColumn id="8" xr3:uid="{CF3B6389-B559-4FE3-8B33-FEDB303382B1}" name="Autumn Week 5" dataDxfId="83"/>
-    <tableColumn id="9" xr3:uid="{8DD80B9C-D1B1-4CDE-A624-4CD3A15113DD}" name="Autumn Week 6" dataDxfId="82"/>
-    <tableColumn id="10" xr3:uid="{8C4EBEE4-01CB-4AD0-B594-F466CC36D370}" name="Autumn Week 7" dataDxfId="81"/>
-    <tableColumn id="11" xr3:uid="{7F8C91DE-BE61-47CF-A916-D06ED7B283E9}" name="Autumn Week 8" dataDxfId="80"/>
-    <tableColumn id="12" xr3:uid="{9D58139A-0F96-4203-8D22-58BC34744B87}" name="Autumn Week 9" dataDxfId="79"/>
-    <tableColumn id="13" xr3:uid="{43C545DF-9B9E-4080-8012-F9EFA0F01283}" name="Autumn Week 10" dataDxfId="78"/>
-    <tableColumn id="14" xr3:uid="{829AB976-2AB2-435C-8F11-DE08DACA4407}" name="Autumn Week 11" dataDxfId="77"/>
-    <tableColumn id="15" xr3:uid="{9126A0EA-FC34-4876-9D56-A0AC39C5526C}" name="Autumn Week 12" dataDxfId="76"/>
-    <tableColumn id="17" xr3:uid="{15B891EE-FCC8-4E53-A90D-3E10FFC1E9FA}" name="Spring Week 1" dataDxfId="75"/>
-    <tableColumn id="18" xr3:uid="{464CA212-3B53-4678-AFE4-8AF8308C1986}" name="Spring Week 2" dataDxfId="74"/>
-    <tableColumn id="19" xr3:uid="{B560E823-CC29-418C-B26C-52D9FFC8C72E}" name="Spring Week 3" dataDxfId="73"/>
-    <tableColumn id="20" xr3:uid="{D95606F3-E0A0-4907-91E0-4AD09D0C65CB}" name="Spring Week 4" dataDxfId="72"/>
-    <tableColumn id="21" xr3:uid="{E71FF892-9A4B-444C-8972-62D92F81B0E7}" name="Spring Week 5" dataDxfId="71"/>
-    <tableColumn id="22" xr3:uid="{C7775BA8-178A-4501-A8DE-2B2CF77A2451}" name="Spring Week 6" dataDxfId="70"/>
-    <tableColumn id="23" xr3:uid="{51A89A97-F839-4F50-88A9-65049D65C9B0}" name="Spring Week 7" dataDxfId="69"/>
-    <tableColumn id="24" xr3:uid="{26EE6D10-4FC4-49AE-8DE6-18AC556C293D}" name="Spring Week 8" dataDxfId="68"/>
-    <tableColumn id="25" xr3:uid="{FCB1B9FB-21DA-415A-86E6-C8E14F864E1B}" name="Spring Week 9" dataDxfId="67"/>
-    <tableColumn id="26" xr3:uid="{54402AE1-DC77-41BA-BCC7-28BCA7186B44}" name="Spring Week 10" dataDxfId="66"/>
-    <tableColumn id="27" xr3:uid="{31C092D1-BD77-4126-8E72-8E74D0D11509}" name="Spring Week 11" dataDxfId="65"/>
-    <tableColumn id="28" xr3:uid="{56D67770-E36A-46FE-97FA-76CD24229C51}" name="Spring Week 12" dataDxfId="64"/>
-    <tableColumn id="38" xr3:uid="{29E08DCE-0D92-40C5-8F33-F1B96FB2F7A4}" name="Spring Exams" dataDxfId="21"/>
-    <tableColumn id="29" xr3:uid="{785AD842-5ED0-4E27-B4B7-26E6FF9AC266}" name="Sub-total" dataDxfId="20">
+    <tableColumn id="32" xr3:uid="{E11C773A-511F-4D25-8636-C56C5B61ED90}" name="Hours" dataDxfId="98"/>
+    <tableColumn id="4" xr3:uid="{04E38F13-8347-412C-866C-6EFE6796253C}" name="Autumn Week 1" dataDxfId="97"/>
+    <tableColumn id="5" xr3:uid="{254D6A24-FC1B-44C7-A3DF-52DA2A250D31}" name="Autumn Week 2" dataDxfId="96"/>
+    <tableColumn id="6" xr3:uid="{9EB326C3-772E-4E56-89FB-BA3A00291293}" name="Autumn Week 3" dataDxfId="95"/>
+    <tableColumn id="7" xr3:uid="{94BC6C78-5A89-4267-B1C1-BFA70E5A9F34}" name="Autumn Week 4" dataDxfId="94"/>
+    <tableColumn id="8" xr3:uid="{CF3B6389-B559-4FE3-8B33-FEDB303382B1}" name="Autumn Week 5" dataDxfId="93"/>
+    <tableColumn id="9" xr3:uid="{8DD80B9C-D1B1-4CDE-A624-4CD3A15113DD}" name="Autumn Week 6" dataDxfId="92"/>
+    <tableColumn id="10" xr3:uid="{8C4EBEE4-01CB-4AD0-B594-F466CC36D370}" name="Autumn Week 7" dataDxfId="91"/>
+    <tableColumn id="11" xr3:uid="{7F8C91DE-BE61-47CF-A916-D06ED7B283E9}" name="Autumn Week 8" dataDxfId="90"/>
+    <tableColumn id="12" xr3:uid="{9D58139A-0F96-4203-8D22-58BC34744B87}" name="Autumn Week 9" dataDxfId="89"/>
+    <tableColumn id="13" xr3:uid="{43C545DF-9B9E-4080-8012-F9EFA0F01283}" name="Autumn Week 10" dataDxfId="88"/>
+    <tableColumn id="14" xr3:uid="{829AB976-2AB2-435C-8F11-DE08DACA4407}" name="Autumn Week 11" dataDxfId="87"/>
+    <tableColumn id="15" xr3:uid="{9126A0EA-FC34-4876-9D56-A0AC39C5526C}" name="Autumn Week 12" dataDxfId="86"/>
+    <tableColumn id="17" xr3:uid="{15B891EE-FCC8-4E53-A90D-3E10FFC1E9FA}" name="Spring Week 1" dataDxfId="85"/>
+    <tableColumn id="18" xr3:uid="{464CA212-3B53-4678-AFE4-8AF8308C1986}" name="Spring Week 2" dataDxfId="84"/>
+    <tableColumn id="19" xr3:uid="{B560E823-CC29-418C-B26C-52D9FFC8C72E}" name="Spring Week 3" dataDxfId="83"/>
+    <tableColumn id="20" xr3:uid="{D95606F3-E0A0-4907-91E0-4AD09D0C65CB}" name="Spring Week 4" dataDxfId="82"/>
+    <tableColumn id="21" xr3:uid="{E71FF892-9A4B-444C-8972-62D92F81B0E7}" name="Spring Week 5" dataDxfId="81"/>
+    <tableColumn id="22" xr3:uid="{C7775BA8-178A-4501-A8DE-2B2CF77A2451}" name="Spring Week 6" dataDxfId="80"/>
+    <tableColumn id="23" xr3:uid="{51A89A97-F839-4F50-88A9-65049D65C9B0}" name="Spring Week 7" dataDxfId="79"/>
+    <tableColumn id="24" xr3:uid="{26EE6D10-4FC4-49AE-8DE6-18AC556C293D}" name="Spring Week 8" dataDxfId="78"/>
+    <tableColumn id="25" xr3:uid="{FCB1B9FB-21DA-415A-86E6-C8E14F864E1B}" name="Spring Week 9" dataDxfId="77"/>
+    <tableColumn id="26" xr3:uid="{54402AE1-DC77-41BA-BCC7-28BCA7186B44}" name="Spring Week 10" dataDxfId="76"/>
+    <tableColumn id="27" xr3:uid="{31C092D1-BD77-4126-8E72-8E74D0D11509}" name="Spring Week 11" dataDxfId="75"/>
+    <tableColumn id="28" xr3:uid="{56D67770-E36A-46FE-97FA-76CD24229C51}" name="Spring Week 12" dataDxfId="74"/>
+    <tableColumn id="38" xr3:uid="{29E08DCE-0D92-40C5-8F33-F1B96FB2F7A4}" name="Spring Exams" dataDxfId="73"/>
+    <tableColumn id="29" xr3:uid="{785AD842-5ED0-4E27-B4B7-26E6FF9AC266}" name="Sub-total" dataDxfId="72">
       <calculatedColumnFormula>SUMIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0",Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="35" xr3:uid="{EE5D0E71-7823-4EE2-9CC1-32BF500AB742}" name="Total Hours" dataDxfId="19">
+    <tableColumn id="35" xr3:uid="{EE5D0E71-7823-4EE2-9CC1-32BF500AB742}" name="Total Hours" dataDxfId="71">
       <calculatedColumnFormula>IF(Table1[[#This Row],[Hours]]&gt;0,Table1[[#This Row],[Hours]],Table1[[#This Row],[Nominal Hours]])*COUNTIF(Table1[[#This Row],[Autumn Week 1]:[Spring Week 12]],"&gt;0")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3908,27 +3908,27 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A071F52D-AD51-4120-94C5-67D4117EBD07}" name="Table14" displayName="Table14" ref="A1:AE64" totalsRowShown="0" headerRowDxfId="63" dataDxfId="61" headerRowBorderDxfId="62" tableBorderDxfId="60" totalsRowBorderDxfId="59">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{A071F52D-AD51-4120-94C5-67D4117EBD07}" name="Table14" displayName="Table14" ref="A1:AE64" totalsRowShown="0" headerRowDxfId="70" dataDxfId="68" headerRowBorderDxfId="69" tableBorderDxfId="67" totalsRowBorderDxfId="66">
   <autoFilter ref="A1:AE64" xr:uid="{FA69A777-C149-48BD-B248-35F32F0AC920}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AD64">
     <sortCondition ref="A1:A132"/>
   </sortState>
   <tableColumns count="31">
-    <tableColumn id="1" xr3:uid="{D7CE4D57-09F4-4B9D-B464-A087075D1C39}" name="Module Code" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{DE2920B2-70AC-48F3-99E7-07B70BC1E928}" name="Module Title" dataDxfId="15">
+    <tableColumn id="1" xr3:uid="{D7CE4D57-09F4-4B9D-B464-A087075D1C39}" name="Module Code" dataDxfId="65"/>
+    <tableColumn id="2" xr3:uid="{DE2920B2-70AC-48F3-99E7-07B70BC1E928}" name="Module Title" dataDxfId="64">
       <calculatedColumnFormula>_xlfn.XLOOKUP(Table14[[#This Row],[Module Code]],Table2[Module Code],Table2[Module Title])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="34" xr3:uid="{55A68E2B-9324-4E9E-9629-6611EC7C904E}" name="Credits" dataDxfId="33">
+    <tableColumn id="34" xr3:uid="{55A68E2B-9324-4E9E-9629-6611EC7C904E}" name="Credits" dataDxfId="63">
       <calculatedColumnFormula>INDEX(Table2[Credits],MATCH(Table14[[#This Row],[Module Code]],Table2[Module Code],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="30" xr3:uid="{9C4C2C35-CE5A-4469-93FA-21FC6F57EDAD}" name="Semester" dataDxfId="32">
+    <tableColumn id="30" xr3:uid="{9C4C2C35-CE5A-4469-93FA-21FC6F57EDAD}" name="Semester" dataDxfId="62">
       <calculatedColumnFormula>INDEX(Table2[Semester],MATCH(Table14[[#This Row],[Module Code]],Table2[Module Code],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="31" xr3:uid="{A7B09E14-0C35-459D-A9D0-5143D8AFFE4E}" name="Nominal Hours" dataDxfId="30">
+    <tableColumn id="31" xr3:uid="{A7B09E14-0C35-459D-A9D0-5143D8AFFE4E}" name="Nominal Hours" dataDxfId="61">
       <calculatedColumnFormula>INDEX(Table2[Contact Time],MATCH(Table14[[#This Row],[Module Code]],Table2[Module Code],0))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{61946E7A-4C82-425B-89A6-3DBD530FCD55}" name="Contact type" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{503822B3-8862-4FCD-9DD3-3B52F57A97BE}" name="Autumn Week 1" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{61946E7A-4C82-425B-89A6-3DBD530FCD55}" name="Contact type" dataDxfId="60"/>
+    <tableColumn id="4" xr3:uid="{503822B3-8862-4FCD-9DD3-3B52F57A97BE}" name="Autumn Week 1" dataDxfId="59"/>
     <tableColumn id="5" xr3:uid="{760391D0-3219-4B11-8E3D-3E00EEDFA9DD}" name="Autumn Week 2" dataDxfId="58"/>
     <tableColumn id="6" xr3:uid="{6EE5E3E9-C4FB-49BE-932C-B84EA0A7970D}" name="Autumn Week 3" dataDxfId="57"/>
     <tableColumn id="7" xr3:uid="{2C7AD515-480E-49A6-8076-95205ACF95EC}" name="Autumn Week 4" dataDxfId="56"/>
@@ -3951,8 +3951,8 @@
     <tableColumn id="25" xr3:uid="{DC35B6C1-904B-4E6A-A04F-ADF850A50D85}" name="Spring Week 9" dataDxfId="39"/>
     <tableColumn id="26" xr3:uid="{BEB9E86A-57BF-4A1E-A499-BADB9EAD1DE9}" name="Spring Week 10" dataDxfId="38"/>
     <tableColumn id="27" xr3:uid="{D640FB81-F093-4E3F-B7A1-6995DDDD6305}" name="Spring Week 11" dataDxfId="37"/>
-    <tableColumn id="28" xr3:uid="{496FDC17-F0F2-4381-96DA-177DC578A786}" name="Spring Week 12" dataDxfId="29"/>
-    <tableColumn id="32" xr3:uid="{65BCC67A-5DC9-4957-BB42-BCF5FCA71B17}" name="Total" dataDxfId="28">
+    <tableColumn id="28" xr3:uid="{496FDC17-F0F2-4381-96DA-177DC578A786}" name="Spring Week 12" dataDxfId="36"/>
+    <tableColumn id="32" xr3:uid="{65BCC67A-5DC9-4957-BB42-BCF5FCA71B17}" name="Total" dataDxfId="35">
       <calculatedColumnFormula>SUM(Table14[[#This Row],[Autumn Week 1]:[Spring Week 12]])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3961,38 +3961,38 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4070B5A2-579F-42D6-AF31-642FC3F016DD}" name="Table2" displayName="Table2" ref="A1:X109" totalsRowShown="0" headerRowDxfId="113" dataDxfId="111" headerRowBorderDxfId="112">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{4070B5A2-579F-42D6-AF31-642FC3F016DD}" name="Table2" displayName="Table2" ref="A1:X109" totalsRowShown="0" headerRowDxfId="34" dataDxfId="32" headerRowBorderDxfId="33">
   <autoFilter ref="A1:X109" xr:uid="{4070B5A2-579F-42D6-AF31-642FC3F016DD}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B64">
     <sortCondition ref="A1:A64"/>
   </sortState>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{A36A2B86-0F30-4188-9ECD-AE5BC71A59F4}" name="Module Code" dataDxfId="110"/>
-    <tableColumn id="2" xr3:uid="{D3F20037-EF35-4207-A530-484E1EB45719}" name="Module Title" dataDxfId="109"/>
-    <tableColumn id="9" xr3:uid="{40C22022-10B9-411F-9B76-B89140ABFFB2}" name="Alternative Module Code" dataDxfId="108"/>
-    <tableColumn id="13" xr3:uid="{CB12E405-1802-457C-AF17-F1B9CB3BBF13}" name="Source" dataDxfId="107"/>
-    <tableColumn id="8" xr3:uid="{EA737976-1AA7-49B6-8752-A388621554F4}" name="Semester" dataDxfId="106"/>
-    <tableColumn id="6" xr3:uid="{16DFC84F-5858-467D-B447-49992D721E4B}" name="Level" dataDxfId="105"/>
-    <tableColumn id="5" xr3:uid="{A17BC4BA-A3CB-442D-9BDC-D3B41B98B389}" name="Credits" dataDxfId="104"/>
-    <tableColumn id="24" xr3:uid="{597B34DA-41F4-4D1D-AA24-07FF8D78D4D2}" name="Parent" dataDxfId="103"/>
-    <tableColumn id="19" xr3:uid="{98846C13-E462-4CFF-858E-AF75931B6712}" name="AllUG" dataDxfId="102"/>
-    <tableColumn id="3" xr3:uid="{7E25B4F4-1A7D-48D9-AAA2-AF5C97240797}" name="Physics" dataDxfId="101"/>
+    <tableColumn id="1" xr3:uid="{A36A2B86-0F30-4188-9ECD-AE5BC71A59F4}" name="Module Code" dataDxfId="31"/>
+    <tableColumn id="2" xr3:uid="{D3F20037-EF35-4207-A530-484E1EB45719}" name="Module Title" dataDxfId="30"/>
+    <tableColumn id="9" xr3:uid="{40C22022-10B9-411F-9B76-B89140ABFFB2}" name="Alternative Module Code" dataDxfId="29"/>
+    <tableColumn id="13" xr3:uid="{CB12E405-1802-457C-AF17-F1B9CB3BBF13}" name="Source" dataDxfId="28"/>
+    <tableColumn id="8" xr3:uid="{EA737976-1AA7-49B6-8752-A388621554F4}" name="Semester" dataDxfId="27"/>
+    <tableColumn id="6" xr3:uid="{16DFC84F-5858-467D-B447-49992D721E4B}" name="Level" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{A17BC4BA-A3CB-442D-9BDC-D3B41B98B389}" name="Credits" dataDxfId="25"/>
+    <tableColumn id="24" xr3:uid="{597B34DA-41F4-4D1D-AA24-07FF8D78D4D2}" name="Parent" dataDxfId="24"/>
+    <tableColumn id="19" xr3:uid="{98846C13-E462-4CFF-858E-AF75931B6712}" name="AllUG" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{7E25B4F4-1A7D-48D9-AAA2-AF5C97240797}" name="Physics" dataDxfId="22"/>
     <tableColumn id="17" xr3:uid="{AA3AE96F-2651-49D7-89AD-BA94806438AE}" name="PhysAstro"/>
-    <tableColumn id="4" xr3:uid="{9C7DD469-E550-411F-8467-246A1543FB38}" name="Astro" dataDxfId="100"/>
-    <tableColumn id="7" xr3:uid="{3C5D3AEB-487E-4678-A42F-BE4BA4D0E9AA}" name="MedPhys" dataDxfId="99"/>
+    <tableColumn id="4" xr3:uid="{9C7DD469-E550-411F-8467-246A1543FB38}" name="Astro" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{3C5D3AEB-487E-4678-A42F-BE4BA4D0E9AA}" name="MedPhys" dataDxfId="20"/>
     <tableColumn id="20" xr3:uid="{C3673B06-C0A2-44F6-8978-F392282CECF8}" name="AllPG"/>
-    <tableColumn id="14" xr3:uid="{AE552873-9B31-41A6-B73C-D052477CA74C}" name="MScPhysics" dataDxfId="98"/>
-    <tableColumn id="15" xr3:uid="{8F51CE76-3A29-487A-A13C-FB63C79CF3E6}" name="MScAstro" dataDxfId="97"/>
-    <tableColumn id="21" xr3:uid="{FC74E264-78AB-4682-A1B8-D8964ED1C3F3}" name="MScDataPhys" dataDxfId="96"/>
-    <tableColumn id="22" xr3:uid="{2D5776F7-D7F7-4D20-A7CB-DB57997AD074}" name="MScDataAstro" dataDxfId="95"/>
+    <tableColumn id="14" xr3:uid="{AE552873-9B31-41A6-B73C-D052477CA74C}" name="MScPhysics" dataDxfId="19"/>
+    <tableColumn id="15" xr3:uid="{8F51CE76-3A29-487A-A13C-FB63C79CF3E6}" name="MScAstro" dataDxfId="18"/>
+    <tableColumn id="21" xr3:uid="{FC74E264-78AB-4682-A1B8-D8964ED1C3F3}" name="MScDataPhys" dataDxfId="17"/>
+    <tableColumn id="22" xr3:uid="{2D5776F7-D7F7-4D20-A7CB-DB57997AD074}" name="MScDataAstro" dataDxfId="16"/>
     <tableColumn id="18" xr3:uid="{10668F71-1EDF-482E-86A5-46E1F3C15120}" name="MScCSPhysics"/>
     <tableColumn id="23" xr3:uid="{E837FCBC-49C7-45CE-AFAA-4F01143EF2A8}" name="CDTCSPhysics"/>
     <tableColumn id="16" xr3:uid="{DB790F5F-BEF0-41CE-A68A-1AA9DF83D66B}" name="Contact Time"/>
-    <tableColumn id="10" xr3:uid="{60774AFA-B365-4EB5-AAFF-6235868F8C97}" name="Exam Weight (%)" dataDxfId="36"/>
-    <tableColumn id="12" xr3:uid="{537B7C75-E9C0-42F2-9F3C-6E960AB2D257}" name="CA weight" dataDxfId="35">
+    <tableColumn id="10" xr3:uid="{60774AFA-B365-4EB5-AAFF-6235868F8C97}" name="Exam Weight (%)" dataDxfId="15"/>
+    <tableColumn id="12" xr3:uid="{537B7C75-E9C0-42F2-9F3C-6E960AB2D257}" name="CA weight" dataDxfId="14">
       <calculatedColumnFormula>100-Table2[[#This Row],[Exam Weight (%)]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{75DA2527-5A08-4ECE-B4E4-752A8F8BF059}" name="CA Check" dataDxfId="34">
+    <tableColumn id="11" xr3:uid="{75DA2527-5A08-4ECE-B4E4-752A8F8BF059}" name="CA Check" dataDxfId="13">
       <calculatedColumnFormula>IF(COUNTIF(Table1[Module Code],Table2[[#This Row],[Module Code]])&gt;0,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Module Code]],Table1[Summative],"Y")*100,SUMIFS(Table1[Sub-total],Table1[Module Code],Table2[[#This Row],[Alternative Module Code]],Table1[Summative],"Y")*100)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -26515,7 +26515,7 @@
       </c>
       <c r="L32" s="6"/>
       <c r="M32" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N32" s="6"/>
       <c r="O32" s="6"/>

</xml_diff>